<commit_message>
Fix: Invalid Type in "Armee" Table + Remove ISO Reference
</commit_message>
<xml_diff>
--- a/Dictionnaire Données 1SGBD Axel NICOLAS.xlsx
+++ b/Dictionnaire Données 1SGBD Axel NICOLAS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AxelT\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\GitHub\1SGBD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB2B7617-4DC9-46CA-A00E-7850797E1CDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AF7F55F-05C9-4804-8F53-190F0350C306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dictionnaire des données" sheetId="1" r:id="rId1"/>
@@ -97,9 +97,6 @@
     <t>3</t>
   </si>
   <si>
-    <t>Code pays (ISO-3)</t>
-  </si>
-  <si>
     <t>Name</t>
   </si>
   <si>
@@ -214,9 +211,6 @@
     <t>2</t>
   </si>
   <si>
-    <t>Code pays alternatif (ISO-2)</t>
-  </si>
-  <si>
     <t>Référence vers la monnaie</t>
   </si>
   <si>
@@ -265,9 +259,6 @@
     <t>TINYINT</t>
   </si>
   <si>
-    <t>Indice de qualité (0-255)</t>
-  </si>
-  <si>
     <t>haveNuclear</t>
   </si>
   <si>
@@ -365,6 +356,15 @@
   </si>
   <si>
     <t>Statut officiel de la langue</t>
+  </si>
+  <si>
+    <t>Code pays</t>
+  </si>
+  <si>
+    <t>Code pays alternatif</t>
+  </si>
+  <si>
+    <t>Indice de qualité (0-100)</t>
   </si>
 </sst>
 </file>
@@ -777,7 +777,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:F70"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
@@ -786,7 +786,7 @@
     <col min="6" max="6" width="74" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:6" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
@@ -795,7 +795,7 @@
       <c r="E2" s="7"/>
       <c r="F2" s="7"/>
     </row>
-    <row r="4" spans="2:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:6" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
         <v>1</v>
       </c>
@@ -804,7 +804,7 @@
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="2:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:6" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>2</v>
       </c>
@@ -821,7 +821,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>7</v>
       </c>
@@ -838,7 +838,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>12</v>
       </c>
@@ -853,7 +853,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>16</v>
       </c>
@@ -868,7 +868,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="2:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:6" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="4" t="s">
         <v>19</v>
       </c>
@@ -877,7 +877,7 @@
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
     </row>
-    <row r="12" spans="2:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:6" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>2</v>
       </c>
@@ -894,7 +894,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
         <v>20</v>
       </c>
@@ -911,7 +911,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
         <v>22</v>
       </c>
@@ -923,87 +923,87 @@
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B15" s="2" t="s">
         <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="2" t="s">
-        <v>26</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B16" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="3" t="s">
         <v>29</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>30</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B17" s="2" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B17" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B18" s="2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="D18" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>37</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B19" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>40</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B20" s="2" t="s">
         <v>41</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>8</v>
@@ -1013,132 +1013,132 @@
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B21" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="2" t="s">
+      <c r="C21" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>44</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>45</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B22" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="2" t="s">
-        <v>47</v>
-      </c>
       <c r="C22" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>37</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B23" s="2" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="C23" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>37</v>
       </c>
       <c r="E23" s="3"/>
       <c r="F23" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B24" s="2" t="s">
         <v>50</v>
-      </c>
-    </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B24" s="2" t="s">
-        <v>51</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B25" s="2" t="s">
         <v>53</v>
-      </c>
-    </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B25" s="2" t="s">
-        <v>54</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E25" s="3"/>
       <c r="F25" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B26" s="2" t="s">
         <v>55</v>
-      </c>
-    </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B26" s="2" t="s">
-        <v>56</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E26" s="3"/>
       <c r="F26" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B27" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B27" s="2" t="s">
+      <c r="C27" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E27" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C27" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E27" s="3" t="s">
+      <c r="F27" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="F27" s="2" t="s">
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B28" s="2" t="s">
         <v>61</v>
-      </c>
-    </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B28" s="2" t="s">
-        <v>62</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E28" s="3"/>
       <c r="F28" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" s="2" t="s">
         <v>7</v>
       </c>
@@ -1149,22 +1149,22 @@
         <v>9</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="32" spans="2:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="5"/>
       <c r="E32" s="5"/>
       <c r="F32" s="5"/>
     </row>
-    <row r="33" spans="2:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:6" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="1" t="s">
         <v>2</v>
       </c>
@@ -1181,9 +1181,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>13</v>
@@ -1195,12 +1195,12 @@
         <v>10</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B35" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>8</v>
@@ -1210,12 +1210,12 @@
       </c>
       <c r="E35" s="3"/>
       <c r="F35" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B36" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>8</v>
@@ -1225,12 +1225,12 @@
       </c>
       <c r="E36" s="3"/>
       <c r="F36" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B37" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>8</v>
@@ -1240,12 +1240,12 @@
       </c>
       <c r="E37" s="3"/>
       <c r="F37" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B38" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>8</v>
@@ -1255,12 +1255,12 @@
       </c>
       <c r="E38" s="3"/>
       <c r="F38" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B39" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>8</v>
@@ -1270,40 +1270,40 @@
       </c>
       <c r="E39" s="3"/>
       <c r="F39" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B40" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C40" s="3" t="s">
         <v>78</v>
-      </c>
-    </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B40" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>80</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E40" s="3"/>
       <c r="F40" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.3">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B41" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E41" s="3"/>
       <c r="F41" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B42" s="2" t="s">
         <v>20</v>
       </c>
@@ -1314,22 +1314,22 @@
         <v>9</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="45" spans="2:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="45" spans="2:6" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5"/>
       <c r="E45" s="5"/>
       <c r="F45" s="5"/>
     </row>
-    <row r="46" spans="2:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:6" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="1" t="s">
         <v>2</v>
       </c>
@@ -1346,9 +1346,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B47" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>8</v>
@@ -1360,10 +1360,10 @@
         <v>10</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B48" s="2" t="s">
         <v>12</v>
       </c>
@@ -1371,16 +1371,16 @@
         <v>23</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="E48" s="3"/>
       <c r="F48" s="2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.3">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="49" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B49" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>23</v>
@@ -1389,30 +1389,30 @@
         <v>24</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="50" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B50" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="E50" s="3"/>
       <c r="F50" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.3">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="51" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B51" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>8</v>
@@ -1422,40 +1422,40 @@
       </c>
       <c r="E51" s="3"/>
       <c r="F51" s="2" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.3">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="52" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B52" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C52" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D52" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="D52" s="3" t="s">
-        <v>37</v>
       </c>
       <c r="E52" s="3"/>
       <c r="F52" s="2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="53" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B53" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C53" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D53" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="D53" s="3" t="s">
-        <v>37</v>
       </c>
       <c r="E53" s="3"/>
       <c r="F53" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B54" s="2" t="s">
         <v>20</v>
       </c>
@@ -1466,22 +1466,22 @@
         <v>9</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="57" spans="2:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="57" spans="2:6" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="4" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C57" s="5"/>
       <c r="D57" s="5"/>
       <c r="E57" s="5"/>
       <c r="F57" s="5"/>
     </row>
-    <row r="58" spans="2:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:6" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="1" t="s">
         <v>2</v>
       </c>
@@ -1498,9 +1498,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B59" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>8</v>
@@ -1512,12 +1512,12 @@
         <v>10</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.3">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="60" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B60" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C60" s="3" t="s">
         <v>23</v>
@@ -1526,58 +1526,58 @@
         <v>24</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="61" spans="2:6" x14ac:dyDescent="0.3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="61" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B61" s="2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E61" s="3"/>
       <c r="F61" s="2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="62" spans="2:6" x14ac:dyDescent="0.3">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="62" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E62" s="3"/>
       <c r="F62" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.3">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="63" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B63" s="2" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="E63" s="3"/>
       <c r="F63" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="64" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B64" s="2" t="s">
         <v>20</v>
       </c>
@@ -1588,22 +1588,22 @@
         <v>9</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="67" spans="2:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="67" spans="2:6" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B67" s="4" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C67" s="5"/>
       <c r="D67" s="5"/>
       <c r="E67" s="5"/>
       <c r="F67" s="5"/>
     </row>
-    <row r="68" spans="2:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:6" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="1" t="s">
         <v>2</v>
       </c>
@@ -1620,7 +1620,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="69" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B69" s="2" t="s">
         <v>20</v>
       </c>
@@ -1631,27 +1631,27 @@
         <v>9</v>
       </c>
       <c r="E69" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="70" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B70" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="F70" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="F69" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="70" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B70" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D70" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E70" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="F70" s="2" t="s">
-        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix: Update all documents for Table Guerre and edit small details in PDF
</commit_message>
<xml_diff>
--- a/Dictionnaire Données 1SGBD Axel NICOLAS.xlsx
+++ b/Dictionnaire Données 1SGBD Axel NICOLAS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\GitHub\1SGBD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AF7F55F-05C9-4804-8F53-190F0350C306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9F9F907-C985-4262-9412-8C8273B4532E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="122">
   <si>
     <t>DICTIONNAIRE DES DONNÉES</t>
   </si>
@@ -365,13 +365,34 @@
   </si>
   <si>
     <t>Indice de qualité (0-100)</t>
+  </si>
+  <si>
+    <t>date_début</t>
+  </si>
+  <si>
+    <t>date_fin</t>
+  </si>
+  <si>
+    <t>DATE</t>
+  </si>
+  <si>
+    <t>statut</t>
+  </si>
+  <si>
+    <t>Statut: en cours, terminée, cessez le feu.</t>
+  </si>
+  <si>
+    <t>Date de fin du conflit (Null si en cours)</t>
+  </si>
+  <si>
+    <t>Date de début du conflit</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -400,6 +421,12 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -776,7 +803,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:F70"/>
+  <dimension ref="B2:F73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -1654,6 +1681,51 @@
         <v>110</v>
       </c>
     </row>
+    <row r="71" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B71" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E71" s="3"/>
+      <c r="F71" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="72" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B72" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E72" s="3"/>
+      <c r="F72" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="73" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B73" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E73" s="3"/>
+      <c r="F73" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="B4:F4"/>
@@ -1664,6 +1736,7 @@
     <mergeCell ref="B32:F32"/>
     <mergeCell ref="B57:F57"/>
   </mergeCells>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>